<commit_message>
Step 1 closed: plan v1.2 approved
Approved by Dan, 2026-08-01, with direction to continue Step 2. v1.2 supersedes v1.0
as the baseline and carries R-01, R-02 and R-03 within it.

Step 1 is closed. Five review rounds produced 28 questions and 3 change requests, all
answered and applied. The baseline is 65 requirements, 21 validation rules and 11
engineering decisions. Any further change now takes the next point release and its own
approval, per the version-control rules on sheet 09.

Both approval rows are recorded on sheet 12: v1.0 (Gate 1) and v1.2 (this issue).

Step 2 continues. The workbook template and dummy data file named in the approval
decision were delivered at v1.1 and remain valid - v1.2 changes no schema.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XSm1KSGtymAaRV3ZhUyDkk
</commit_message>
<xml_diff>
--- a/docs/PRAP_Development_Plan_v1.2.xlsx
+++ b/docs/PRAP_Development_Plan_v1.2.xlsx
@@ -145,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -188,9 +188,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -556,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B89"/>
+  <dimension ref="A1:B88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -597,7 +594,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Development plan (Step 1 deliverable) - change against the v1.0 baseline</t>
+          <t>Development plan (Step 1 deliverable) - approved baseline</t>
         </is>
       </c>
     </row>
@@ -621,7 +618,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Change against approved baseline v1.0 - R-03 confirmed, ready for approval</t>
+          <t>APPROVED BASELINE - approved by Dan 2026-08-01, supersedes v1.0</t>
         </is>
       </c>
     </row>
@@ -664,12 +661,12 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Baseline</t>
+          <t>Approved by</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>v1.0, approved by Dan 2026-08-01 (Gate 1)</t>
+          <t>Dan, 2026-08-01 - this issue is now the baseline</t>
         </is>
       </c>
     </row>
@@ -705,7 +702,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>v1.1 (draft, never approved). v1.0 remains the approved baseline until this issue is approved</t>
+          <t>v1.0 (approved 2026-08-01) and v1.1 (draft)</t>
         </is>
       </c>
     </row>
@@ -864,374 +861,367 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>Nothing in this document is open. Five review rounds produced 28 questions and 3 change requests; all</t>
+          <t>APPROVED by Dan on 2026-08-01. This issue is the baseline, superseding v1.0. Five review rounds</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>31 are answered and applied. The only outstanding item is the approval signature on sheet 12 for this</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <t>change against the v1.0 baseline.</t>
+          <t>produced 28 questions and 3 change requests; all 31 are answered and applied, and Step 1 is closed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>The plan in one page</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t>The plan in one page</t>
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Output        One HTML file, opened by double-click on Windows, offline, no install. One Excel</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Output        One HTML file, opened by double-click on Windows, offline, no install. One Excel</t>
+          <t xml:space="preserve">                workbook alongside it holds the data and remains the archive of record.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                workbook alongside it holds the data and remains the archive of record.</t>
-        </is>
-      </c>
+      <c r="A46" s="6" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="inlineStr"/>
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Calculation   load = project period weight x role factor x person weight x month coverage,</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Calculation   load = project period weight x role factor x person weight x month coverage,</t>
+          <t xml:space="preserve">                in FTE where 1.00 FTE = 160 hours per month.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">                in FTE where 1.00 FTE = 160 hours per month.</t>
+          <t xml:space="preserve">                Over-allocated above 1.50 FTE in a month; under-allocated below 0.80 FTE for three</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">                Over-allocated above 1.50 FTE in a month; under-allocated below 0.80 FTE for three</t>
+          <t xml:space="preserve">                or more consecutive months, reported as a run.</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                or more consecutive months, reported as a run.</t>
-        </is>
-      </c>
+      <c r="A51" s="6" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="6" t="inlineStr"/>
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Periods       Clinical Trial: five period names derived from milestone dates and month offsets,</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Periods       Clinical Trial: five period names derived from milestone dates and month offsets,</t>
+          <t xml:space="preserve">                with Conduct occurring up to twice where an interim DB lock splits it. Weights come</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">                with Conduct occurring up to twice where an interim DB lock splits it. Weights come</t>
+          <t xml:space="preserve">                from the trial's clinical phase.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">                from the trial's clinical phase.</t>
+          <t xml:space="preserve">                Others: three periods, dates and weights both entered by hand.</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                Others: three periods, dates and weights both entered by hand.</t>
-        </is>
-      </c>
+      <c r="A56" s="6" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="6" t="inlineStr"/>
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Dashboard     Overall (monthly simulation per project and per person, tables and graphs),</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Dashboard     Overall (monthly simulation per project and per person, tables and graphs),</t>
+          <t xml:space="preserve">                Source data (project), Source data (person). Every field editable, with identifier</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">                Source data (project), Source data (person). Every field editable, with identifier</t>
+          <t xml:space="preserve">                edits cascading to referencing rows.</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                edits cascading to referencing rows.</t>
-        </is>
-      </c>
+      <c r="A60" s="6" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="6" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="6" t="inlineStr">
+      <c r="A61" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Build         Five steps, each ending at a review gate. This document closes Step 1.</t>
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>What approving this document means</t>
+        </is>
+      </c>
+    </row>
     <row r="64">
-      <c r="A64" s="5" t="inlineStr">
-        <is>
-          <t>What approving this document means</t>
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>Gate 1 approval on sheet 12 baselines the 63 requirements on sheet 03 as the contract for Steps 2-5,</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>Gate 1 approval on sheet 12 baselines the 63 requirements on sheet 03 as the contract for Steps 2-5,</t>
+          <t>and confirms the six engineering decisions C-06 to C-11 on sheet 05 that were proposed but never</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>and confirms the six engineering decisions C-06 to C-11 on sheet 05 that were proposed but never</t>
+          <t>explicitly answered across the review rounds. Those six are listed there with their rationale; if any</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>explicitly answered across the review rounds. Those six are listed there with their rationale; if any</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="6" t="inlineStr">
-        <is>
           <t>is wrong, say so at approval rather than after.</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="5" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
         <is>
           <t>How to read this workbook</t>
         </is>
       </c>
     </row>
-    <row r="71" ht="28" customHeight="1">
-      <c r="A71" s="7" t="inlineStr">
+    <row r="70" ht="28" customHeight="1">
+      <c r="A70" s="7" t="inlineStr">
         <is>
           <t>Sheet</t>
         </is>
       </c>
-      <c r="B71" s="7" t="inlineStr">
+      <c r="B70" s="7" t="inlineStr">
         <is>
           <t>Contents</t>
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" s="8" t="inlineStr">
+        <is>
+          <t>00_Cover</t>
+        </is>
+      </c>
+      <c r="B71" s="9" t="inlineStr">
+        <is>
+          <t>Document control, what changed, reading guide.</t>
+        </is>
+      </c>
+    </row>
     <row r="72">
-      <c r="A72" s="8" t="inlineStr">
-        <is>
-          <t>00_Cover</t>
-        </is>
-      </c>
-      <c r="B72" s="9" t="inlineStr">
-        <is>
-          <t>Document control, what changed, reading guide.</t>
+      <c r="A72" s="10" t="inlineStr">
+        <is>
+          <t>01_Version_History</t>
+        </is>
+      </c>
+      <c r="B72" s="11" t="inlineStr">
+        <is>
+          <t>Change log for this plan.</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="10" t="inlineStr">
-        <is>
-          <t>01_Version_History</t>
-        </is>
-      </c>
-      <c r="B73" s="11" t="inlineStr">
-        <is>
-          <t>Change log for this plan.</t>
+      <c r="A73" s="8" t="inlineStr">
+        <is>
+          <t>02_Scope</t>
+        </is>
+      </c>
+      <c r="B73" s="9" t="inlineStr">
+        <is>
+          <t>Background, objectives, in scope / out of scope.</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="8" t="inlineStr">
-        <is>
-          <t>02_Scope</t>
-        </is>
-      </c>
-      <c r="B74" s="9" t="inlineStr">
-        <is>
-          <t>Background, objectives, in scope / out of scope.</t>
+      <c r="A74" s="10" t="inlineStr">
+        <is>
+          <t>03_Requirements</t>
+        </is>
+      </c>
+      <c r="B74" s="11" t="inlineStr">
+        <is>
+          <t>Numbered requirement register - the contract for Steps 2-5.</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="10" t="inlineStr">
-        <is>
-          <t>03_Requirements</t>
-        </is>
-      </c>
-      <c r="B75" s="11" t="inlineStr">
-        <is>
-          <t>Numbered requirement register - the contract for Steps 2-5.</t>
+      <c r="A75" s="8" t="inlineStr">
+        <is>
+          <t>04_Data_Model</t>
+        </is>
+      </c>
+      <c r="B75" s="9" t="inlineStr">
+        <is>
+          <t>Every sheet and column of the single source workbook, with rules.</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="8" t="inlineStr">
-        <is>
-          <t>04_Data_Model</t>
-        </is>
-      </c>
-      <c r="B76" s="9" t="inlineStr">
-        <is>
-          <t>Every sheet and column of the single source workbook, with rules.</t>
+      <c r="A76" s="10" t="inlineStr">
+        <is>
+          <t>05_Resource_Logic</t>
+        </is>
+      </c>
+      <c r="B76" s="11" t="inlineStr">
+        <is>
+          <t>The calculation that turns assignments and weights into monthly FTE.</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="10" t="inlineStr">
-        <is>
-          <t>05_Resource_Logic</t>
-        </is>
-      </c>
-      <c r="B77" s="11" t="inlineStr">
-        <is>
-          <t>The calculation that turns assignments and weights into monthly FTE.</t>
+      <c r="A77" s="8" t="inlineStr">
+        <is>
+          <t>06_Dashboard_Design</t>
+        </is>
+      </c>
+      <c r="B77" s="9" t="inlineStr">
+        <is>
+          <t>The three dashboard tabs: tables, graphs, filters, editing.</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="8" t="inlineStr">
-        <is>
-          <t>06_Dashboard_Design</t>
-        </is>
-      </c>
-      <c r="B78" s="9" t="inlineStr">
-        <is>
-          <t>The three dashboard tabs: tables, graphs, filters, editing.</t>
+      <c r="A78" s="10" t="inlineStr">
+        <is>
+          <t>07_Architecture</t>
+        </is>
+      </c>
+      <c r="B78" s="11" t="inlineStr">
+        <is>
+          <t>Single-file HTML + Excel-on-disk design and the file-access decision.</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="10" t="inlineStr">
-        <is>
-          <t>07_Architecture</t>
-        </is>
-      </c>
-      <c r="B79" s="11" t="inlineStr">
-        <is>
-          <t>Single-file HTML + Excel-on-disk design and the file-access decision.</t>
+      <c r="A79" s="8" t="inlineStr">
+        <is>
+          <t>08_WBS_Schedule</t>
+        </is>
+      </c>
+      <c r="B79" s="9" t="inlineStr">
+        <is>
+          <t>The five steps broken into tasks, deliverables and review gates.</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="8" t="inlineStr">
-        <is>
-          <t>08_WBS_Schedule</t>
-        </is>
-      </c>
-      <c r="B80" s="9" t="inlineStr">
-        <is>
-          <t>The five steps broken into tasks, deliverables and review gates.</t>
+      <c r="A80" s="10" t="inlineStr">
+        <is>
+          <t>09_Version_Control</t>
+        </is>
+      </c>
+      <c r="B80" s="11" t="inlineStr">
+        <is>
+          <t>How plan, specification and output files are versioned together.</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="10" t="inlineStr">
-        <is>
-          <t>09_Version_Control</t>
-        </is>
-      </c>
-      <c r="B81" s="11" t="inlineStr">
-        <is>
-          <t>How plan, specification and output files are versioned together.</t>
+      <c r="A81" s="8" t="inlineStr">
+        <is>
+          <t>10_Risks</t>
+        </is>
+      </c>
+      <c r="B81" s="9" t="inlineStr">
+        <is>
+          <t>Risks and assumptions with mitigations.</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="8" t="inlineStr">
-        <is>
-          <t>10_Risks</t>
-        </is>
-      </c>
-      <c r="B82" s="9" t="inlineStr">
-        <is>
-          <t>Risks and assumptions with mitigations.</t>
+      <c r="A82" s="10" t="inlineStr">
+        <is>
+          <t>11_Open_Questions</t>
+        </is>
+      </c>
+      <c r="B82" s="11" t="inlineStr">
+        <is>
+          <t>All 28 questions and their answers. Nothing open.</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="10" t="inlineStr">
-        <is>
-          <t>11_Open_Questions</t>
-        </is>
-      </c>
-      <c r="B83" s="11" t="inlineStr">
-        <is>
-          <t>All 28 questions and their answers. Nothing open.</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="8" t="inlineStr">
+      <c r="A83" s="8" t="inlineStr">
         <is>
           <t>12_Review_Log</t>
         </is>
       </c>
-      <c r="B84" s="9" t="inlineStr">
+      <c r="B83" s="9" t="inlineStr">
         <is>
           <t>Every change made across the four review rounds, and why. Gate 1 approval block.</t>
         </is>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>Legend</t>
+        </is>
+      </c>
+    </row>
     <row r="86">
-      <c r="A86" s="3" t="inlineStr">
-        <is>
-          <t>Legend</t>
+      <c r="A86" s="12" t="inlineStr">
+        <is>
+          <t>Green = new in v0.2, added from your review answers.</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="12" t="inlineStr">
-        <is>
-          <t>Green = new in v0.2, added from your review answers.</t>
+      <c r="A87" s="13" t="inlineStr">
+        <is>
+          <t>Orange = changed in v0.2 as a consequence of your review.</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="13" t="inlineStr">
-        <is>
-          <t>Orange = changed in v0.2 as a consequence of your review.</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="14" t="inlineStr">
+      <c r="A88" s="14" t="inlineStr">
         <is>
           <t>Yellow = still needs your input.</t>
         </is>
@@ -1785,7 +1775,7 @@
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>R-03 confirmed. Awaiting the approval signature.</t>
+          <t>APPROVED 2026-08-01 by Dan. Current baseline. Step 1 closed.</t>
         </is>
       </c>
     </row>
@@ -5025,23 +5015,31 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="10" t="inlineStr">
+      <c r="A56" s="20" t="inlineStr">
         <is>
           <t>PRAP Development Plan v1.2</t>
         </is>
       </c>
-      <c r="B56" s="22" t="inlineStr"/>
-      <c r="C56" s="22" t="inlineStr"/>
-      <c r="D56" s="11" t="inlineStr">
-        <is>
-          <t>Pending your signature. Change against the v1.0 baseline: R-01, R-02 and R-03 all applied and confirmed. Nothing outstanding in the document itself.</t>
+      <c r="B56" s="20" t="inlineStr">
+        <is>
+          <t>Dan</t>
+        </is>
+      </c>
+      <c r="C56" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D56" s="19" t="inlineStr">
+        <is>
+          <t>APPROVED. Finalise plan v1.2 and continue Step 2. This issue supersedes v1.0 as the baseline; R-01, R-02 and R-03 are part of it.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="16" t="inlineStr">
         <is>
-          <t>GATE 1 PASSED at v1.0: the requirements on sheet 03 are baselined as the contract for Steps 2-5 and decisions C-06 to C-11 are confirmed. v1.1 is a change against that baseline and needs the second approval above before it supersedes v1.0. Step 2 continues in the meantime - the change affects the period derivation and the milestone list, both of which are data the application reads.</t>
+          <t>STEP 1 CLOSED. v1.2 is the approved baseline: the 65 requirements on sheet 03 are the contract for Steps 2-5, and decisions C-01 to C-11 on sheet 05 are confirmed. Any further change takes the next point release and its own approval, per the rules on sheet 09.</t>
         </is>
       </c>
     </row>
@@ -5525,12 +5523,12 @@
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>R-03 confirmed and closed. No content change beyond recording it: the derivation, requirements and validation rules are as issued at v1.1. Every question and change request raised across five review rounds is now settled, and the only outstanding item is the approval signature for this change.</t>
+          <t>R-03 confirmed and closed. No content change beyond recording it: the derivation, requirements and validation rules are as issued at v1.1. Every question and change request raised across five review rounds is now settled.</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>For approval</t>
+          <t>APPROVED 2026-08-01 by Dan - baseline</t>
         </is>
       </c>
     </row>
@@ -13518,7 +13516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -13916,7 +13914,7 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>Pending you</t>
+          <t>Complete</t>
         </is>
       </c>
     </row>
@@ -13928,12 +13926,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>G1b</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>GATE 1 - development plan approved by Dan, 2026-08-01. Decisions C-06..C-11 confirmed.</t>
+          <t>GATE 1 RE-CONFIRMED - plan v1.2 approved by Dan, 2026-08-01. Step 1 closed.</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -13950,27 +13948,27 @@
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Generate the source workbook template and a dummy data file for review.</t>
+          <t>GATE 1 - development plan approved by Dan, 2026-08-01. Decisions C-06..C-11 confirmed.</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>PRAP_SourceData_Template + _Dummy v1.1</t>
+          <t>Approval recorded on 12_Review_Log</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>Complete - issued for review</t>
+          <t>Complete</t>
         </is>
       </c>
     </row>
@@ -13982,22 +13980,22 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Fix the source workbook schema: exact sheet names, column headers, types, value lists.</t>
+          <t>Generate the source workbook template and a dummy data file for review.</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Specification sheet 'Data schema'</t>
+          <t>PRAP_SourceData_Template + _Dummy v1.1</t>
         </is>
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Complete - issued for review</t>
         </is>
       </c>
     </row>
@@ -14009,22 +14007,22 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>Specify the calculation engine as pseudocode plus the worked example as an acceptance test.</t>
+          <t>Fix the source workbook schema: exact sheet names, column headers, types, value lists.</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Specification sheet 'Calculation'</t>
+          <t>Specification sheet 'Data schema'</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
     </row>
@@ -14036,12 +14034,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Specify period derivation per project type, and the over/under-allocation detection.</t>
+          <t>Specify the calculation engine as pseudocode plus the worked example as an acceptance test.</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -14063,17 +14061,17 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>Specify import validation rules V-01..V-21 and the findings report.</t>
+          <t>Specify period derivation per project type, and the over/under-allocation detection.</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>Specification sheet 'Validation'</t>
+          <t>Specification sheet 'Calculation'</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -14090,17 +14088,17 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Specify each dashboard tab: every table, column, graph, filter and interaction.</t>
+          <t>Specify import validation rules V-01..V-21 and the findings report.</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Specification sheet 'UI spec'</t>
+          <t>Specification sheet 'Validation'</t>
         </is>
       </c>
       <c r="E24" s="10" t="inlineStr">
@@ -14117,17 +14115,17 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>2.6</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>Specify on-screen editing, the dirty-state model and export round-tripping.</t>
+          <t>Specify each dashboard tab: every table, column, graph, filter and interaction.</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>Specification sheet 'Editing &amp; IO'</t>
+          <t>Specification sheet 'UI spec'</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -14144,17 +14142,17 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>2.7</t>
+          <t>2.6</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Specify the version/compatibility check.</t>
+          <t>Specify on-screen editing, the dirty-state model and export round-tripping.</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Specification sheet 'IO &amp; versioning'</t>
+          <t>Specification sheet 'Editing &amp; IO'</t>
         </is>
       </c>
       <c r="E26" s="10" t="inlineStr">
@@ -14171,17 +14169,17 @@
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>2.7</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>Build the requirement-to-specification traceability matrix.</t>
+          <t>Specify the version/compatibility check.</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Specification sheet 'Traceability'</t>
+          <t>Specification sheet 'IO &amp; versioning'</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
@@ -14198,17 +14196,17 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>G2</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>GATE 2 - programming specification approved.</t>
+          <t>Build the requirement-to-specification traceability matrix.</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>PRAP_Programming_Specification_v1.0.xlsx</t>
+          <t>Specification sheet 'Traceability'</t>
         </is>
       </c>
       <c r="E28" s="10" t="inlineStr">
@@ -14220,22 +14218,22 @@
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>G2</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>High-level UI design: tab structure, page regions, navigation. No code behind it.</t>
+          <t>GATE 2 - programming specification approved.</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Prototype HTML (UI only)</t>
+          <t>PRAP_Programming_Specification_v1.0.xlsx</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
@@ -14252,17 +14250,17 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Requester reviews the high-level component design.</t>
+          <t>High-level UI design: tab structure, page regions, navigation. No code behind it.</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Review comments</t>
+          <t>Prototype HTML (UI only)</t>
         </is>
       </c>
       <c r="E30" s="10" t="inlineStr">
@@ -14279,17 +14277,17 @@
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>Final UI design with clear per-component requirements.</t>
+          <t>Requester reviews the high-level component design.</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Prototype HTML v1.0 + component list</t>
+          <t>Review comments</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -14306,17 +14304,17 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>G3</t>
+          <t>3.3</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>GATE 3 - final design and component list approved. Code generation starts only for approved components.</t>
+          <t>Final UI design with clear per-component requirements.</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Approved component list</t>
+          <t>Prototype HTML v1.0 + component list</t>
         </is>
       </c>
       <c r="E32" s="10" t="inlineStr">
@@ -14328,22 +14326,22 @@
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>G3</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>IO layer: workbook load, sheet/column mapping, export.</t>
+          <t>GATE 3 - final design and component list approved. Code generation starts only for approved components.</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Application code</t>
+          <t>Approved component list</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
@@ -14360,12 +14358,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Validation layer: rules V-01..V-21 and the findings report.</t>
+          <t>IO layer: workbook load, sheet/column mapping, export.</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -14387,12 +14385,12 @@
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>Model layer, Lists and Config handling.</t>
+          <t>Validation layer: rules V-01..V-21 and the findings report.</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
@@ -14414,12 +14412,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Edit buffer: on-screen editing, dirty state, per-edit validation.</t>
+          <t>Model layer, Lists and Config handling.</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -14441,17 +14439,17 @@
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.4</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>Calculation engine, verified against the worked example.</t>
+          <t>Edit buffer: on-screen editing, dirty state, per-edit validation.</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Application code + test evidence</t>
+          <t>Application code</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
@@ -14468,17 +14466,17 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Overall tab: tables, graphs, filters, over/under-allocation flagging.</t>
+          <t>Calculation engine, verified against the worked example.</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Application code</t>
+          <t>Application code + test evidence</t>
         </is>
       </c>
       <c r="E38" s="10" t="inlineStr">
@@ -14495,12 +14493,12 @@
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>Source data (project) and Source data (person) tabs.</t>
+          <t>Overall tab: tables, graphs, filters, over/under-allocation flagging.</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
@@ -14522,17 +14520,17 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Blank source workbook template with value lists and example rows.</t>
+          <t>Source data (project) and Source data (person) tabs.</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>PRAP_SourceData template</t>
+          <t>Application code</t>
         </is>
       </c>
       <c r="E40" s="10" t="inlineStr">
@@ -14549,17 +14547,17 @@
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>Requester reviews output against real data; refinements folded in.</t>
+          <t>Blank source workbook template with value lists and example rows.</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>Updated code</t>
+          <t>PRAP_SourceData template</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
@@ -14576,17 +14574,17 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>4.9</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>GATE 4 - application functionally complete.</t>
+          <t>Requester reviews output against real data; refinements folded in.</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>PRAP_Application_v0.9.html</t>
+          <t>Updated code</t>
         </is>
       </c>
       <c r="E42" s="10" t="inlineStr">
@@ -14598,22 +14596,22 @@
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>G4</t>
         </is>
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>Full pass over the traceability matrix: every Must requirement demonstrated.</t>
+          <t>GATE 4 - application functionally complete.</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>Completed traceability matrix</t>
+          <t>PRAP_Application_v0.9.html</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
@@ -14630,17 +14628,17 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>5.2</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Test on a clean Windows PC in Edge and Chrome, offline.</t>
+          <t>Full pass over the traceability matrix: every Must requirement demonstrated.</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Test evidence</t>
+          <t>Completed traceability matrix</t>
         </is>
       </c>
       <c r="E44" s="10" t="inlineStr">
@@ -14657,17 +14655,17 @@
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>5.3</t>
+          <t>5.2</t>
         </is>
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>Write the user guide: folder layout, how to load, how to maintain source data.</t>
+          <t>Test on a clean Windows PC in Edge and Chrome, offline.</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>User guide</t>
+          <t>Test evidence</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
@@ -14684,17 +14682,17 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>5.4</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Final version alignment across plan, specification and application.</t>
+          <t>Write the user guide: folder layout, how to load, how to maintain source data.</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Version alignment table (sheet 09)</t>
+          <t>User guide</t>
         </is>
       </c>
       <c r="E46" s="10" t="inlineStr">
@@ -14711,90 +14709,117 @@
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
+          <t>5.4</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>Final version alignment across plan, specification and application.</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>Version alignment table (sheet 09)</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B48" s="10" t="inlineStr">
+        <is>
           <t>G5</t>
         </is>
       </c>
-      <c r="C47" s="9" t="inlineStr">
+      <c r="C48" s="11" t="inlineStr">
         <is>
           <t>GATE 5 - release.</t>
         </is>
       </c>
-      <c r="D47" s="9" t="inlineStr">
+      <c r="D48" s="11" t="inlineStr">
         <is>
           <t>PRAP_Application_v1.0.html</t>
         </is>
       </c>
-      <c r="E47" s="8" t="inlineStr">
+      <c r="E48" s="10" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>Progress</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="28" customHeight="1">
-      <c r="A50" s="7" t="inlineStr">
+    <row r="51" ht="28" customHeight="1">
+      <c r="A51" s="7" t="inlineStr">
         <is>
           <t>Measure</t>
         </is>
       </c>
-      <c r="B50" s="7" t="inlineStr">
+      <c r="B51" s="7" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>Tasks total</t>
         </is>
       </c>
-      <c r="B51" s="8">
-        <f>COUNTA(B5:B47)</f>
+      <c r="B52" s="8">
+        <f>COUNTA(B5:B48)</f>
         <v/>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="10" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="10" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="B52" s="10">
-        <f>COUNTIF(E5:E47,"Complete")+COUNTIF(E5:E47,"Complete - issued for review")</f>
+      <c r="B53" s="10">
+        <f>COUNTIF(E5:E48,"Complete")+COUNTIF(E5:E48,"Complete - issued for review")</f>
         <v/>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="8" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>Awaiting the requester</t>
         </is>
       </c>
-      <c r="B53" s="8">
-        <f>COUNTIF(E5:E47,"Pending you")</f>
+      <c r="B54" s="8">
+        <f>COUNTIF(E5:E48,"Pending you")</f>
         <v/>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="10" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="10" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="B54" s="10">
-        <f>COUNTIF(E5:E47,"Not started")</f>
+      <c r="B55" s="10">
+        <f>COUNTIF(E5:E48,"Not started")</f>
         <v/>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="16" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="16" t="inlineStr">
         <is>
           <t>No duration estimates: the pace is set by review turnaround at each gate, not by build effort.</t>
         </is>
@@ -14802,7 +14827,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="E5:E47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E5:E48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,In progress,Pending you,Complete - issued for review,Complete,Blocked"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>